<commit_message>
Update 05 Chemische Parameter.xlsx
</commit_message>
<xml_diff>
--- a/Wasser/05 Chemische Parameter.xlsx
+++ b/Wasser/05 Chemische Parameter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexandra\Documents\2. Uni\Master\Masterarbeit\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alexandra\Documents\GitHub\Moore-Lichtenau-Meusebach\Wasser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70CDEAD-B679-4C84-BD4B-B9FD9FF772C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7C8C55-FDFD-4573-9E14-B6FA5A8FA65B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{C748F3ED-3D32-4CFF-8258-545184BF166B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{C748F3ED-3D32-4CFF-8258-545184BF166B}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Meusebach trocken" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1101" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="105">
   <si>
     <t xml:space="preserve">Datum </t>
   </si>
@@ -512,7 +512,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -522,12 +522,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-4.9989318521683403E-2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1049,7 +1043,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1184,27 +1178,99 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1214,21 +1280,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1238,18 +1289,6 @@
     <xf numFmtId="14" fontId="2" fillId="2" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1276,81 +1315,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="38" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1728,40 +1692,40 @@
       <c r="B3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="57" t="s">
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="59"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="80"/>
+      <c r="S3" s="80"/>
+      <c r="T3" s="81"/>
     </row>
     <row r="4" spans="1:20" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="77" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="C4" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="62"/>
+      <c r="D4" s="76"/>
       <c r="E4" s="2" t="s">
         <v>45</v>
       </c>
@@ -1783,10 +1747,10 @@
       <c r="K4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="61" t="s">
+      <c r="L4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M4" s="62"/>
+      <c r="M4" s="76"/>
       <c r="N4" s="7" t="s">
         <v>45</v>
       </c>
@@ -1810,47 +1774,47 @@
       </c>
     </row>
     <row r="5" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60"/>
+      <c r="A5" s="77"/>
       <c r="B5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="63">
-        <v>0</v>
-      </c>
-      <c r="D5" s="64"/>
+      <c r="C5" s="78">
+        <v>0</v>
+      </c>
+      <c r="D5" s="74"/>
       <c r="E5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F5" s="29"/>
-      <c r="G5" s="64">
-        <v>0</v>
-      </c>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="G5" s="74">
+        <v>0</v>
+      </c>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
       <c r="J5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K5" s="30"/>
-      <c r="L5" s="63">
-        <v>0</v>
-      </c>
-      <c r="M5" s="64"/>
+      <c r="L5" s="78">
+        <v>0</v>
+      </c>
+      <c r="M5" s="74"/>
       <c r="N5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O5" s="29"/>
-      <c r="P5" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="64"/>
-      <c r="R5" s="64"/>
+      <c r="P5" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="74"/>
+      <c r="R5" s="74"/>
       <c r="S5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T5" s="30"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="60"/>
+      <c r="A6" s="77"/>
       <c r="B6" s="23" t="s">
         <v>10</v>
       </c>
@@ -1910,7 +1874,7 @@
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="60"/>
+      <c r="A7" s="77"/>
       <c r="B7" s="23" t="s">
         <v>8</v>
       </c>
@@ -1946,7 +1910,7 @@
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="60"/>
+      <c r="A8" s="77"/>
       <c r="B8" s="23" t="s">
         <v>37</v>
       </c>
@@ -2000,7 +1964,7 @@
       </c>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A9" s="60"/>
+      <c r="A9" s="77"/>
       <c r="B9" s="23" t="s">
         <v>9</v>
       </c>
@@ -2030,7 +1994,7 @@
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A10" s="60"/>
+      <c r="A10" s="77"/>
       <c r="B10" s="24" t="s">
         <v>32</v>
       </c>
@@ -2074,16 +2038,16 @@
       </c>
     </row>
     <row r="11" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+      <c r="A11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="62"/>
+      <c r="D11" s="76"/>
       <c r="E11" s="2" t="s">
         <v>45</v>
       </c>
@@ -2105,10 +2069,10 @@
       <c r="K11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="61" t="s">
+      <c r="L11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M11" s="62"/>
+      <c r="M11" s="76"/>
       <c r="N11" s="7" t="s">
         <v>45</v>
       </c>
@@ -2132,47 +2096,47 @@
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A12" s="60"/>
+      <c r="A12" s="77"/>
       <c r="B12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="63">
-        <v>0</v>
-      </c>
-      <c r="D12" s="64"/>
+      <c r="C12" s="78">
+        <v>0</v>
+      </c>
+      <c r="D12" s="74"/>
       <c r="E12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F12" s="29"/>
-      <c r="G12" s="64">
-        <v>0</v>
-      </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
+      <c r="G12" s="74">
+        <v>0</v>
+      </c>
+      <c r="H12" s="74"/>
+      <c r="I12" s="74"/>
       <c r="J12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K12" s="30"/>
-      <c r="L12" s="63">
-        <v>0</v>
-      </c>
-      <c r="M12" s="64"/>
+      <c r="L12" s="78">
+        <v>0</v>
+      </c>
+      <c r="M12" s="74"/>
       <c r="N12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O12" s="29"/>
-      <c r="P12" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="64"/>
-      <c r="R12" s="64"/>
+      <c r="P12" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
       <c r="S12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T12" s="30"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A13" s="60"/>
+      <c r="A13" s="77"/>
       <c r="B13" s="23" t="s">
         <v>10</v>
       </c>
@@ -2232,7 +2196,7 @@
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A14" s="60"/>
+      <c r="A14" s="77"/>
       <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
@@ -2268,7 +2232,7 @@
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A15" s="60"/>
+      <c r="A15" s="77"/>
       <c r="B15" s="23" t="s">
         <v>37</v>
       </c>
@@ -2322,7 +2286,7 @@
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A16" s="60"/>
+      <c r="A16" s="77"/>
       <c r="B16" s="23" t="s">
         <v>9</v>
       </c>
@@ -2352,7 +2316,7 @@
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A17" s="60"/>
+      <c r="A17" s="77"/>
       <c r="B17" s="24" t="s">
         <v>32</v>
       </c>
@@ -2396,16 +2360,16 @@
       </c>
     </row>
     <row r="18" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="60" t="s">
+      <c r="A18" s="77" t="s">
         <v>72</v>
       </c>
       <c r="B18" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="62"/>
+      <c r="D18" s="76"/>
       <c r="E18" s="2" t="s">
         <v>45</v>
       </c>
@@ -2427,10 +2391,10 @@
       <c r="K18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="61" t="s">
+      <c r="L18" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="M18" s="62"/>
+      <c r="M18" s="76"/>
       <c r="N18" s="7" t="s">
         <v>45</v>
       </c>
@@ -2454,47 +2418,47 @@
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A19" s="60"/>
+      <c r="A19" s="77"/>
       <c r="B19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="63">
-        <v>0</v>
-      </c>
-      <c r="D19" s="64"/>
+      <c r="C19" s="78">
+        <v>0</v>
+      </c>
+      <c r="D19" s="74"/>
       <c r="E19" s="40" t="s">
         <v>46</v>
       </c>
       <c r="F19" s="29"/>
-      <c r="G19" s="64">
-        <v>0</v>
-      </c>
-      <c r="H19" s="64"/>
-      <c r="I19" s="64"/>
+      <c r="G19" s="74">
+        <v>0</v>
+      </c>
+      <c r="H19" s="74"/>
+      <c r="I19" s="74"/>
       <c r="J19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K19" s="30"/>
-      <c r="L19" s="63">
-        <v>0</v>
-      </c>
-      <c r="M19" s="64"/>
+      <c r="L19" s="78">
+        <v>0</v>
+      </c>
+      <c r="M19" s="74"/>
       <c r="N19" s="40" t="s">
         <v>46</v>
       </c>
       <c r="O19" s="29"/>
-      <c r="P19" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="64"/>
-      <c r="R19" s="64"/>
+      <c r="P19" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
       <c r="S19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T19" s="30"/>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A20" s="60"/>
+      <c r="A20" s="77"/>
       <c r="B20" s="23" t="s">
         <v>10</v>
       </c>
@@ -2554,7 +2518,7 @@
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A21" s="60"/>
+      <c r="A21" s="77"/>
       <c r="B21" s="23" t="s">
         <v>8</v>
       </c>
@@ -2590,7 +2554,7 @@
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A22" s="60"/>
+      <c r="A22" s="77"/>
       <c r="B22" s="23" t="s">
         <v>37</v>
       </c>
@@ -2644,7 +2608,7 @@
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A23" s="60"/>
+      <c r="A23" s="77"/>
       <c r="B23" s="23" t="s">
         <v>9</v>
       </c>
@@ -2674,7 +2638,7 @@
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A24" s="60"/>
+      <c r="A24" s="77"/>
       <c r="B24" s="24" t="s">
         <v>32</v>
       </c>
@@ -2718,16 +2682,16 @@
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="77" t="s">
         <v>86</v>
       </c>
       <c r="B25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="75" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="62"/>
+      <c r="D25" s="76"/>
       <c r="E25" s="2" t="s">
         <v>45</v>
       </c>
@@ -2749,10 +2713,10 @@
       <c r="K25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L25" s="61" t="s">
+      <c r="L25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M25" s="62"/>
+      <c r="M25" s="76"/>
       <c r="N25" s="7" t="s">
         <v>45</v>
       </c>
@@ -2776,47 +2740,47 @@
       </c>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A26" s="60"/>
+      <c r="A26" s="77"/>
       <c r="B26" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="63">
-        <v>0</v>
-      </c>
-      <c r="D26" s="64"/>
+      <c r="C26" s="78">
+        <v>0</v>
+      </c>
+      <c r="D26" s="74"/>
       <c r="E26" s="40" t="s">
         <v>46</v>
       </c>
       <c r="F26" s="29"/>
-      <c r="G26" s="64">
-        <v>0</v>
-      </c>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
+      <c r="G26" s="74">
+        <v>0</v>
+      </c>
+      <c r="H26" s="74"/>
+      <c r="I26" s="74"/>
       <c r="J26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K26" s="30"/>
-      <c r="L26" s="63">
-        <v>0</v>
-      </c>
-      <c r="M26" s="64"/>
+      <c r="L26" s="78">
+        <v>0</v>
+      </c>
+      <c r="M26" s="74"/>
       <c r="N26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O26" s="29"/>
-      <c r="P26" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="64"/>
-      <c r="R26" s="64"/>
+      <c r="P26" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
       <c r="S26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T26" s="30"/>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A27" s="60"/>
+      <c r="A27" s="77"/>
       <c r="B27" s="23" t="s">
         <v>10</v>
       </c>
@@ -2876,7 +2840,7 @@
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A28" s="60"/>
+      <c r="A28" s="77"/>
       <c r="B28" s="23" t="s">
         <v>8</v>
       </c>
@@ -2912,7 +2876,7 @@
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A29" s="60"/>
+      <c r="A29" s="77"/>
       <c r="B29" s="23" t="s">
         <v>37</v>
       </c>
@@ -2966,7 +2930,7 @@
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A30" s="60"/>
+      <c r="A30" s="77"/>
       <c r="B30" s="23" t="s">
         <v>9</v>
       </c>
@@ -2996,7 +2960,7 @@
       </c>
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A31" s="60"/>
+      <c r="A31" s="77"/>
       <c r="B31" s="24" t="s">
         <v>32</v>
       </c>
@@ -3046,20 +3010,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="A18:A24"/>
-    <mergeCell ref="P26:R26"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="G26:I26"/>
     <mergeCell ref="C3:K3"/>
     <mergeCell ref="L3:T3"/>
     <mergeCell ref="A25:A31"/>
@@ -3076,6 +3026,20 @@
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A11:A17"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A18:A24"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="0.11811023622047245" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -3144,57 +3108,57 @@
       <c r="B3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="57" t="s">
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="59"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="80"/>
+      <c r="S3" s="80"/>
+      <c r="T3" s="81"/>
       <c r="U3" s="31" t="s">
         <v>0</v>
       </c>
       <c r="V3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="W3" s="57" t="s">
+      <c r="W3" s="79" t="s">
         <v>7</v>
       </c>
-      <c r="X3" s="58"/>
-      <c r="Y3" s="58"/>
-      <c r="Z3" s="58"/>
-      <c r="AA3" s="58"/>
-      <c r="AB3" s="58"/>
-      <c r="AC3" s="58"/>
-      <c r="AD3" s="58"/>
-      <c r="AE3" s="59"/>
+      <c r="X3" s="80"/>
+      <c r="Y3" s="80"/>
+      <c r="Z3" s="80"/>
+      <c r="AA3" s="80"/>
+      <c r="AB3" s="80"/>
+      <c r="AC3" s="80"/>
+      <c r="AD3" s="80"/>
+      <c r="AE3" s="81"/>
     </row>
     <row r="4" spans="1:32" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="77" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="C4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="62"/>
+      <c r="D4" s="76"/>
       <c r="E4" s="2" t="s">
         <v>45</v>
       </c>
@@ -3216,10 +3180,10 @@
       <c r="K4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="61" t="s">
+      <c r="L4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M4" s="62"/>
+      <c r="M4" s="76"/>
       <c r="N4" s="2" t="s">
         <v>45</v>
       </c>
@@ -3241,16 +3205,16 @@
       <c r="T4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="60" t="s">
+      <c r="U4" s="77" t="s">
         <v>50</v>
       </c>
       <c r="V4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W4" s="61" t="s">
+      <c r="W4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X4" s="62"/>
+      <c r="X4" s="76"/>
       <c r="Y4" s="7" t="s">
         <v>45</v>
       </c>
@@ -3274,68 +3238,68 @@
       </c>
     </row>
     <row r="5" spans="1:32" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60"/>
+      <c r="A5" s="77"/>
       <c r="B5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="63">
-        <v>0</v>
-      </c>
-      <c r="D5" s="64"/>
+      <c r="C5" s="78">
+        <v>0</v>
+      </c>
+      <c r="D5" s="74"/>
       <c r="E5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F5" s="29"/>
-      <c r="G5" s="64">
-        <v>0</v>
-      </c>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="G5" s="74">
+        <v>0</v>
+      </c>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
       <c r="J5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K5" s="30"/>
-      <c r="L5" s="63">
-        <v>0</v>
-      </c>
-      <c r="M5" s="64"/>
+      <c r="L5" s="78">
+        <v>0</v>
+      </c>
+      <c r="M5" s="74"/>
       <c r="N5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O5" s="29"/>
-      <c r="P5" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="64"/>
-      <c r="R5" s="64"/>
+      <c r="P5" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="74"/>
+      <c r="R5" s="74"/>
       <c r="S5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T5" s="30"/>
-      <c r="U5" s="60"/>
+      <c r="U5" s="77"/>
       <c r="V5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W5" s="63">
-        <v>0</v>
-      </c>
-      <c r="X5" s="64"/>
+      <c r="W5" s="78">
+        <v>0</v>
+      </c>
+      <c r="X5" s="74"/>
       <c r="Y5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z5" s="29"/>
-      <c r="AA5" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="64"/>
-      <c r="AC5" s="64"/>
+      <c r="AA5" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="74"/>
+      <c r="AC5" s="74"/>
       <c r="AD5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE5" s="30"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A6" s="60"/>
+      <c r="A6" s="77"/>
       <c r="B6" s="23" t="s">
         <v>10</v>
       </c>
@@ -3393,7 +3357,7 @@
       <c r="T6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U6" s="60"/>
+      <c r="U6" s="77"/>
       <c r="V6" s="23" t="s">
         <v>10</v>
       </c>
@@ -3426,7 +3390,7 @@
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A7" s="60"/>
+      <c r="A7" s="77"/>
       <c r="B7" s="23" t="s">
         <v>8</v>
       </c>
@@ -3460,7 +3424,7 @@
       <c r="T7" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U7" s="60"/>
+      <c r="U7" s="77"/>
       <c r="V7" s="23" t="s">
         <v>8</v>
       </c>
@@ -3481,7 +3445,7 @@
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A8" s="60"/>
+      <c r="A8" s="77"/>
       <c r="B8" s="23" t="s">
         <v>37</v>
       </c>
@@ -3533,7 +3497,7 @@
       <c r="T8" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U8" s="60"/>
+      <c r="U8" s="77"/>
       <c r="V8" s="23" t="s">
         <v>37</v>
       </c>
@@ -3563,7 +3527,7 @@
       </c>
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A9" s="60"/>
+      <c r="A9" s="77"/>
       <c r="B9" s="23" t="s">
         <v>9</v>
       </c>
@@ -3591,7 +3555,7 @@
       <c r="T9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U9" s="60"/>
+      <c r="U9" s="77"/>
       <c r="V9" s="23" t="s">
         <v>9</v>
       </c>
@@ -3609,7 +3573,7 @@
       </c>
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A10" s="60"/>
+      <c r="A10" s="77"/>
       <c r="B10" s="24" t="s">
         <v>32</v>
       </c>
@@ -3651,7 +3615,7 @@
       <c r="T10" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U10" s="60"/>
+      <c r="U10" s="77"/>
       <c r="V10" s="24" t="s">
         <v>32</v>
       </c>
@@ -3676,16 +3640,16 @@
       </c>
     </row>
     <row r="11" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+      <c r="A11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="62"/>
+      <c r="D11" s="76"/>
       <c r="E11" s="7" t="s">
         <v>45</v>
       </c>
@@ -3707,10 +3671,10 @@
       <c r="K11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="61" t="s">
+      <c r="L11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M11" s="62"/>
+      <c r="M11" s="76"/>
       <c r="N11" s="7" t="s">
         <v>45</v>
       </c>
@@ -3732,16 +3696,16 @@
       <c r="T11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U11" s="60" t="s">
+      <c r="U11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="V11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W11" s="61" t="s">
+      <c r="W11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X11" s="62"/>
+      <c r="X11" s="76"/>
       <c r="Y11" s="7" t="s">
         <v>45</v>
       </c>
@@ -3768,68 +3732,68 @@
       </c>
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A12" s="60"/>
+      <c r="A12" s="77"/>
       <c r="B12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="63">
-        <v>0</v>
-      </c>
-      <c r="D12" s="64"/>
+      <c r="C12" s="78">
+        <v>0</v>
+      </c>
+      <c r="D12" s="74"/>
       <c r="E12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F12" s="29"/>
-      <c r="G12" s="64">
-        <v>0</v>
-      </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
+      <c r="G12" s="74">
+        <v>0</v>
+      </c>
+      <c r="H12" s="74"/>
+      <c r="I12" s="74"/>
       <c r="J12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K12" s="30"/>
-      <c r="L12" s="63">
-        <v>0</v>
-      </c>
-      <c r="M12" s="64"/>
+      <c r="L12" s="78">
+        <v>0</v>
+      </c>
+      <c r="M12" s="74"/>
       <c r="N12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O12" s="29"/>
-      <c r="P12" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="64"/>
-      <c r="R12" s="64"/>
+      <c r="P12" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
       <c r="S12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T12" s="30"/>
-      <c r="U12" s="60"/>
+      <c r="U12" s="77"/>
       <c r="V12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W12" s="63">
-        <v>0</v>
-      </c>
-      <c r="X12" s="64"/>
+      <c r="W12" s="78">
+        <v>0</v>
+      </c>
+      <c r="X12" s="74"/>
       <c r="Y12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z12" s="29"/>
-      <c r="AA12" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="64"/>
-      <c r="AC12" s="64"/>
+      <c r="AA12" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="74"/>
+      <c r="AC12" s="74"/>
       <c r="AD12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE12" s="30"/>
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A13" s="60"/>
+      <c r="A13" s="77"/>
       <c r="B13" s="23" t="s">
         <v>10</v>
       </c>
@@ -3887,7 +3851,7 @@
       <c r="T13" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U13" s="60"/>
+      <c r="U13" s="77"/>
       <c r="V13" s="23" t="s">
         <v>10</v>
       </c>
@@ -3920,7 +3884,7 @@
       </c>
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A14" s="60"/>
+      <c r="A14" s="77"/>
       <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
@@ -3954,7 +3918,7 @@
       <c r="T14" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U14" s="60"/>
+      <c r="U14" s="77"/>
       <c r="V14" s="23" t="s">
         <v>8</v>
       </c>
@@ -3975,7 +3939,7 @@
       </c>
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A15" s="60"/>
+      <c r="A15" s="77"/>
       <c r="B15" s="23" t="s">
         <v>37</v>
       </c>
@@ -4027,7 +3991,7 @@
       <c r="T15" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U15" s="60"/>
+      <c r="U15" s="77"/>
       <c r="V15" s="23" t="s">
         <v>37</v>
       </c>
@@ -4057,7 +4021,7 @@
       </c>
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A16" s="60"/>
+      <c r="A16" s="77"/>
       <c r="B16" s="23" t="s">
         <v>9</v>
       </c>
@@ -4085,7 +4049,7 @@
       <c r="T16" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U16" s="60"/>
+      <c r="U16" s="77"/>
       <c r="V16" s="23" t="s">
         <v>9</v>
       </c>
@@ -4103,7 +4067,7 @@
       </c>
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A17" s="60"/>
+      <c r="A17" s="77"/>
       <c r="B17" s="24" t="s">
         <v>32</v>
       </c>
@@ -4145,7 +4109,7 @@
       <c r="T17" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U17" s="60"/>
+      <c r="U17" s="77"/>
       <c r="V17" s="24" t="s">
         <v>32</v>
       </c>
@@ -4170,16 +4134,16 @@
       </c>
     </row>
     <row r="18" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="60" t="s">
+      <c r="A18" s="77" t="s">
         <v>72</v>
       </c>
       <c r="B18" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="62"/>
+      <c r="D18" s="76"/>
       <c r="E18" s="7" t="s">
         <v>45</v>
       </c>
@@ -4201,10 +4165,10 @@
       <c r="K18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="61" t="s">
+      <c r="L18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M18" s="62"/>
+      <c r="M18" s="76"/>
       <c r="N18" s="7" t="s">
         <v>45</v>
       </c>
@@ -4226,16 +4190,16 @@
       <c r="T18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U18" s="60" t="s">
+      <c r="U18" s="77" t="s">
         <v>72</v>
       </c>
       <c r="V18" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W18" s="61" t="s">
+      <c r="W18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X18" s="62"/>
+      <c r="X18" s="76"/>
       <c r="Y18" s="7" t="s">
         <v>45</v>
       </c>
@@ -4259,68 +4223,68 @@
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A19" s="60"/>
+      <c r="A19" s="77"/>
       <c r="B19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="63">
-        <v>0</v>
-      </c>
-      <c r="D19" s="64"/>
+      <c r="C19" s="78">
+        <v>0</v>
+      </c>
+      <c r="D19" s="74"/>
       <c r="E19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F19" s="29"/>
-      <c r="G19" s="64">
-        <v>0</v>
-      </c>
-      <c r="H19" s="64"/>
-      <c r="I19" s="64"/>
+      <c r="G19" s="74">
+        <v>0</v>
+      </c>
+      <c r="H19" s="74"/>
+      <c r="I19" s="74"/>
       <c r="J19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K19" s="30"/>
-      <c r="L19" s="63">
-        <v>0</v>
-      </c>
-      <c r="M19" s="64"/>
+      <c r="L19" s="78">
+        <v>0</v>
+      </c>
+      <c r="M19" s="74"/>
       <c r="N19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O19" s="29"/>
-      <c r="P19" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="64"/>
-      <c r="R19" s="64"/>
+      <c r="P19" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
       <c r="S19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T19" s="30"/>
-      <c r="U19" s="60"/>
+      <c r="U19" s="77"/>
       <c r="V19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W19" s="63">
-        <v>0</v>
-      </c>
-      <c r="X19" s="64"/>
+      <c r="W19" s="78">
+        <v>0</v>
+      </c>
+      <c r="X19" s="74"/>
       <c r="Y19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z19" s="29"/>
-      <c r="AA19" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="64"/>
-      <c r="AC19" s="64"/>
+      <c r="AA19" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="74"/>
+      <c r="AC19" s="74"/>
       <c r="AD19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE19" s="30"/>
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A20" s="60"/>
+      <c r="A20" s="77"/>
       <c r="B20" s="23" t="s">
         <v>10</v>
       </c>
@@ -4378,7 +4342,7 @@
       <c r="T20" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U20" s="60"/>
+      <c r="U20" s="77"/>
       <c r="V20" s="23" t="s">
         <v>10</v>
       </c>
@@ -4411,7 +4375,7 @@
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A21" s="60"/>
+      <c r="A21" s="77"/>
       <c r="B21" s="23" t="s">
         <v>8</v>
       </c>
@@ -4445,7 +4409,7 @@
       <c r="T21" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U21" s="60"/>
+      <c r="U21" s="77"/>
       <c r="V21" s="23" t="s">
         <v>8</v>
       </c>
@@ -4466,7 +4430,7 @@
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A22" s="60"/>
+      <c r="A22" s="77"/>
       <c r="B22" s="23" t="s">
         <v>37</v>
       </c>
@@ -4518,7 +4482,7 @@
       <c r="T22" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U22" s="60"/>
+      <c r="U22" s="77"/>
       <c r="V22" s="23" t="s">
         <v>37</v>
       </c>
@@ -4548,7 +4512,7 @@
       </c>
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A23" s="60"/>
+      <c r="A23" s="77"/>
       <c r="B23" s="23" t="s">
         <v>9</v>
       </c>
@@ -4576,7 +4540,7 @@
       <c r="T23" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U23" s="60"/>
+      <c r="U23" s="77"/>
       <c r="V23" s="23" t="s">
         <v>9</v>
       </c>
@@ -4594,7 +4558,7 @@
       </c>
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A24" s="60"/>
+      <c r="A24" s="77"/>
       <c r="B24" s="24" t="s">
         <v>32</v>
       </c>
@@ -4636,7 +4600,7 @@
       <c r="T24" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U24" s="60"/>
+      <c r="U24" s="77"/>
       <c r="V24" s="24" t="s">
         <v>32</v>
       </c>
@@ -4661,16 +4625,16 @@
       </c>
     </row>
     <row r="25" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="65" t="s">
+      <c r="A25" s="82" t="s">
         <v>86</v>
       </c>
       <c r="B25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="62"/>
+      <c r="D25" s="76"/>
       <c r="E25" s="7" t="s">
         <v>45</v>
       </c>
@@ -4692,33 +4656,41 @@
       <c r="K25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L25" s="68"/>
-      <c r="M25" s="69"/>
-      <c r="N25" s="49" t="s">
+      <c r="L25" s="75" t="s">
+        <v>48</v>
+      </c>
+      <c r="M25" s="76"/>
+      <c r="N25" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="O25" s="50"/>
-      <c r="P25" s="48" t="s">
+      <c r="O25" s="41">
+        <v>0</v>
+      </c>
+      <c r="P25" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="Q25" s="51"/>
-      <c r="R25" s="48" t="s">
+      <c r="Q25" s="41">
+        <v>0</v>
+      </c>
+      <c r="R25" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="S25" s="51"/>
-      <c r="T25" s="48" t="s">
+      <c r="S25" s="41">
+        <v>0</v>
+      </c>
+      <c r="T25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U25" s="60" t="s">
+      <c r="U25" s="77" t="s">
         <v>86</v>
       </c>
       <c r="V25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W25" s="61" t="s">
+      <c r="W25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X25" s="62"/>
+      <c r="X25" s="76"/>
       <c r="Y25" s="7" t="s">
         <v>45</v>
       </c>
@@ -4742,64 +4714,68 @@
       </c>
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A26" s="66"/>
+      <c r="A26" s="83"/>
       <c r="B26" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="63">
-        <v>0</v>
-      </c>
-      <c r="D26" s="64"/>
+      <c r="C26" s="78">
+        <v>0</v>
+      </c>
+      <c r="D26" s="74"/>
       <c r="E26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F26" s="29"/>
-      <c r="G26" s="64">
-        <v>0</v>
-      </c>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
+      <c r="G26" s="74">
+        <v>0</v>
+      </c>
+      <c r="H26" s="74"/>
+      <c r="I26" s="74"/>
       <c r="J26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K26" s="30"/>
-      <c r="L26" s="70"/>
-      <c r="M26" s="71"/>
-      <c r="N26" s="52" t="s">
+      <c r="L26" s="78">
+        <v>0</v>
+      </c>
+      <c r="M26" s="74"/>
+      <c r="N26" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="O26" s="29"/>
+      <c r="P26" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
+      <c r="S26" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="O26" s="53"/>
-      <c r="P26" s="71"/>
-      <c r="Q26" s="71"/>
-      <c r="R26" s="71"/>
-      <c r="S26" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="T26" s="55"/>
-      <c r="U26" s="60"/>
+      <c r="T26" s="30"/>
+      <c r="U26" s="77"/>
       <c r="V26" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W26" s="63">
-        <v>0</v>
-      </c>
-      <c r="X26" s="64"/>
+      <c r="W26" s="78">
+        <v>0</v>
+      </c>
+      <c r="X26" s="74"/>
       <c r="Y26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z26" s="29"/>
-      <c r="AA26" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="64"/>
-      <c r="AC26" s="64"/>
+      <c r="AA26" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="74"/>
+      <c r="AC26" s="74"/>
       <c r="AD26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE26" s="30"/>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A27" s="66"/>
+      <c r="A27" s="83"/>
       <c r="B27" s="23" t="s">
         <v>10</v>
       </c>
@@ -4857,7 +4833,7 @@
       <c r="T27" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U27" s="60"/>
+      <c r="U27" s="77"/>
       <c r="V27" s="23" t="s">
         <v>10</v>
       </c>
@@ -4890,7 +4866,7 @@
       </c>
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A28" s="66"/>
+      <c r="A28" s="83"/>
       <c r="B28" s="23" t="s">
         <v>8</v>
       </c>
@@ -4924,7 +4900,7 @@
       <c r="T28" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U28" s="60"/>
+      <c r="U28" s="77"/>
       <c r="V28" s="23" t="s">
         <v>8</v>
       </c>
@@ -4945,7 +4921,7 @@
       </c>
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A29" s="66"/>
+      <c r="A29" s="83"/>
       <c r="B29" s="23" t="s">
         <v>37</v>
       </c>
@@ -4997,7 +4973,7 @@
       <c r="T29" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U29" s="60"/>
+      <c r="U29" s="77"/>
       <c r="V29" s="23" t="s">
         <v>37</v>
       </c>
@@ -5027,7 +5003,7 @@
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A30" s="66"/>
+      <c r="A30" s="83"/>
       <c r="B30" s="23" t="s">
         <v>9</v>
       </c>
@@ -5055,7 +5031,7 @@
       <c r="T30" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U30" s="60"/>
+      <c r="U30" s="77"/>
       <c r="V30" s="23" t="s">
         <v>9</v>
       </c>
@@ -5073,7 +5049,7 @@
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A31" s="67"/>
+      <c r="A31" s="84"/>
       <c r="B31" s="24" t="s">
         <v>32</v>
       </c>
@@ -5115,7 +5091,7 @@
       <c r="T31" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U31" s="60"/>
+      <c r="U31" s="77"/>
       <c r="V31" s="24" t="s">
         <v>32</v>
       </c>
@@ -5146,15 +5122,28 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="W25:X25"/>
-    <mergeCell ref="W26:X26"/>
-    <mergeCell ref="AA26:AC26"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="W12:X12"/>
-    <mergeCell ref="AA12:AC12"/>
-    <mergeCell ref="W18:X18"/>
-    <mergeCell ref="W19:X19"/>
-    <mergeCell ref="AA19:AC19"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="C3:K3"/>
+    <mergeCell ref="L3:T3"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="W3:AE3"/>
+    <mergeCell ref="A4:A10"/>
+    <mergeCell ref="U4:U10"/>
+    <mergeCell ref="W4:X4"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="AA5:AC5"/>
     <mergeCell ref="A18:A24"/>
     <mergeCell ref="U18:U24"/>
     <mergeCell ref="A25:A31"/>
@@ -5171,28 +5160,15 @@
     <mergeCell ref="L12:M12"/>
     <mergeCell ref="P12:R12"/>
     <mergeCell ref="L18:M18"/>
-    <mergeCell ref="W3:AE3"/>
-    <mergeCell ref="A4:A10"/>
-    <mergeCell ref="U4:U10"/>
-    <mergeCell ref="W4:X4"/>
-    <mergeCell ref="W5:X5"/>
-    <mergeCell ref="AA5:AC5"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="C3:K3"/>
-    <mergeCell ref="L3:T3"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="P26:R26"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="W25:X25"/>
+    <mergeCell ref="W26:X26"/>
+    <mergeCell ref="AA26:AC26"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="W12:X12"/>
+    <mergeCell ref="AA12:AC12"/>
+    <mergeCell ref="W18:X18"/>
+    <mergeCell ref="W19:X19"/>
+    <mergeCell ref="AA19:AC19"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="0.11811023622047245" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -5273,68 +5249,68 @@
       <c r="B3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="59"/>
-      <c r="L3" s="57" t="s">
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="81"/>
+      <c r="L3" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="58"/>
-      <c r="T3" s="59"/>
+      <c r="M3" s="80"/>
+      <c r="N3" s="80"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="80"/>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="80"/>
+      <c r="S3" s="80"/>
+      <c r="T3" s="81"/>
       <c r="U3" s="31" t="s">
         <v>0</v>
       </c>
       <c r="V3" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="W3" s="57" t="s">
+      <c r="W3" s="79" t="s">
         <v>7</v>
       </c>
-      <c r="X3" s="58"/>
-      <c r="Y3" s="58"/>
-      <c r="Z3" s="58"/>
-      <c r="AA3" s="58"/>
-      <c r="AB3" s="58"/>
-      <c r="AC3" s="58"/>
-      <c r="AD3" s="58"/>
-      <c r="AE3" s="59"/>
-      <c r="AF3" s="57" t="s">
+      <c r="X3" s="80"/>
+      <c r="Y3" s="80"/>
+      <c r="Z3" s="80"/>
+      <c r="AA3" s="80"/>
+      <c r="AB3" s="80"/>
+      <c r="AC3" s="80"/>
+      <c r="AD3" s="80"/>
+      <c r="AE3" s="81"/>
+      <c r="AF3" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="AG3" s="58"/>
-      <c r="AH3" s="58"/>
-      <c r="AI3" s="58"/>
-      <c r="AJ3" s="58"/>
-      <c r="AK3" s="58"/>
-      <c r="AL3" s="58"/>
-      <c r="AM3" s="58"/>
-      <c r="AN3" s="59"/>
+      <c r="AG3" s="80"/>
+      <c r="AH3" s="80"/>
+      <c r="AI3" s="80"/>
+      <c r="AJ3" s="80"/>
+      <c r="AK3" s="80"/>
+      <c r="AL3" s="80"/>
+      <c r="AM3" s="80"/>
+      <c r="AN3" s="81"/>
     </row>
     <row r="4" spans="1:40" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="60" t="s">
+      <c r="A4" s="77" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="61" t="s">
+      <c r="C4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="62"/>
+      <c r="D4" s="76"/>
       <c r="E4" s="2" t="s">
         <v>45</v>
       </c>
@@ -5356,10 +5332,10 @@
       <c r="K4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="61" t="s">
+      <c r="L4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M4" s="62"/>
+      <c r="M4" s="76"/>
       <c r="N4" s="7" t="s">
         <v>45</v>
       </c>
@@ -5381,16 +5357,16 @@
       <c r="T4" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="U4" s="60" t="s">
+      <c r="U4" s="77" t="s">
         <v>50</v>
       </c>
       <c r="V4" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W4" s="61" t="s">
+      <c r="W4" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X4" s="62"/>
+      <c r="X4" s="76"/>
       <c r="Y4" s="2" t="s">
         <v>45</v>
       </c>
@@ -5412,90 +5388,90 @@
       <c r="AE4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="AF4" s="72" t="s">
+      <c r="AF4" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="AG4" s="73"/>
-      <c r="AH4" s="73"/>
-      <c r="AI4" s="73"/>
-      <c r="AJ4" s="73"/>
-      <c r="AK4" s="73"/>
-      <c r="AL4" s="73"/>
-      <c r="AM4" s="73"/>
-      <c r="AN4" s="74"/>
+      <c r="AG4" s="86"/>
+      <c r="AH4" s="86"/>
+      <c r="AI4" s="86"/>
+      <c r="AJ4" s="86"/>
+      <c r="AK4" s="86"/>
+      <c r="AL4" s="86"/>
+      <c r="AM4" s="86"/>
+      <c r="AN4" s="87"/>
     </row>
     <row r="5" spans="1:40" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="60"/>
+      <c r="A5" s="77"/>
       <c r="B5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="63">
-        <v>0</v>
-      </c>
-      <c r="D5" s="64"/>
+      <c r="C5" s="78">
+        <v>0</v>
+      </c>
+      <c r="D5" s="74"/>
       <c r="E5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F5" s="29"/>
-      <c r="G5" s="64">
-        <v>0</v>
-      </c>
-      <c r="H5" s="64"/>
-      <c r="I5" s="64"/>
+      <c r="G5" s="74">
+        <v>0</v>
+      </c>
+      <c r="H5" s="74"/>
+      <c r="I5" s="74"/>
       <c r="J5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K5" s="30"/>
-      <c r="L5" s="63">
-        <v>0</v>
-      </c>
-      <c r="M5" s="64"/>
+      <c r="L5" s="78">
+        <v>0</v>
+      </c>
+      <c r="M5" s="74"/>
       <c r="N5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O5" s="29"/>
-      <c r="P5" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="64"/>
-      <c r="R5" s="64"/>
+      <c r="P5" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="74"/>
+      <c r="R5" s="74"/>
       <c r="S5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T5" s="30"/>
-      <c r="U5" s="60"/>
+      <c r="U5" s="77"/>
       <c r="V5" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W5" s="63">
-        <v>0</v>
-      </c>
-      <c r="X5" s="64"/>
+      <c r="W5" s="78">
+        <v>0</v>
+      </c>
+      <c r="X5" s="74"/>
       <c r="Y5" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z5" s="29"/>
-      <c r="AA5" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB5" s="64"/>
-      <c r="AC5" s="64"/>
+      <c r="AA5" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="74"/>
+      <c r="AC5" s="74"/>
       <c r="AD5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE5" s="30"/>
-      <c r="AF5" s="75"/>
-      <c r="AG5" s="76"/>
-      <c r="AH5" s="76"/>
-      <c r="AI5" s="76"/>
-      <c r="AJ5" s="76"/>
-      <c r="AK5" s="76"/>
-      <c r="AL5" s="76"/>
-      <c r="AM5" s="76"/>
-      <c r="AN5" s="77"/>
+      <c r="AF5" s="88"/>
+      <c r="AG5" s="89"/>
+      <c r="AH5" s="89"/>
+      <c r="AI5" s="89"/>
+      <c r="AJ5" s="89"/>
+      <c r="AK5" s="89"/>
+      <c r="AL5" s="89"/>
+      <c r="AM5" s="89"/>
+      <c r="AN5" s="90"/>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A6" s="60"/>
+      <c r="A6" s="77"/>
       <c r="B6" s="23" t="s">
         <v>10</v>
       </c>
@@ -5553,7 +5529,7 @@
       <c r="T6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U6" s="60"/>
+      <c r="U6" s="77"/>
       <c r="V6" s="23" t="s">
         <v>10</v>
       </c>
@@ -5584,18 +5560,18 @@
       <c r="AE6" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF6" s="75"/>
-      <c r="AG6" s="76"/>
-      <c r="AH6" s="76"/>
-      <c r="AI6" s="76"/>
-      <c r="AJ6" s="76"/>
-      <c r="AK6" s="76"/>
-      <c r="AL6" s="76"/>
-      <c r="AM6" s="76"/>
-      <c r="AN6" s="77"/>
+      <c r="AF6" s="88"/>
+      <c r="AG6" s="89"/>
+      <c r="AH6" s="89"/>
+      <c r="AI6" s="89"/>
+      <c r="AJ6" s="89"/>
+      <c r="AK6" s="89"/>
+      <c r="AL6" s="89"/>
+      <c r="AM6" s="89"/>
+      <c r="AN6" s="90"/>
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A7" s="60"/>
+      <c r="A7" s="77"/>
       <c r="B7" s="23" t="s">
         <v>8</v>
       </c>
@@ -5629,7 +5605,7 @@
       <c r="T7" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U7" s="60"/>
+      <c r="U7" s="77"/>
       <c r="V7" s="23" t="s">
         <v>8</v>
       </c>
@@ -5648,18 +5624,18 @@
       <c r="AE7" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF7" s="75"/>
-      <c r="AG7" s="76"/>
-      <c r="AH7" s="76"/>
-      <c r="AI7" s="76"/>
-      <c r="AJ7" s="76"/>
-      <c r="AK7" s="76"/>
-      <c r="AL7" s="76"/>
-      <c r="AM7" s="76"/>
-      <c r="AN7" s="77"/>
+      <c r="AF7" s="88"/>
+      <c r="AG7" s="89"/>
+      <c r="AH7" s="89"/>
+      <c r="AI7" s="89"/>
+      <c r="AJ7" s="89"/>
+      <c r="AK7" s="89"/>
+      <c r="AL7" s="89"/>
+      <c r="AM7" s="89"/>
+      <c r="AN7" s="90"/>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A8" s="60"/>
+      <c r="A8" s="77"/>
       <c r="B8" s="23" t="s">
         <v>37</v>
       </c>
@@ -5711,7 +5687,7 @@
       <c r="T8" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U8" s="60"/>
+      <c r="U8" s="77"/>
       <c r="V8" s="23" t="s">
         <v>37</v>
       </c>
@@ -5739,18 +5715,18 @@
       <c r="AE8" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF8" s="75"/>
-      <c r="AG8" s="76"/>
-      <c r="AH8" s="76"/>
-      <c r="AI8" s="76"/>
-      <c r="AJ8" s="76"/>
-      <c r="AK8" s="76"/>
-      <c r="AL8" s="76"/>
-      <c r="AM8" s="76"/>
-      <c r="AN8" s="77"/>
+      <c r="AF8" s="88"/>
+      <c r="AG8" s="89"/>
+      <c r="AH8" s="89"/>
+      <c r="AI8" s="89"/>
+      <c r="AJ8" s="89"/>
+      <c r="AK8" s="89"/>
+      <c r="AL8" s="89"/>
+      <c r="AM8" s="89"/>
+      <c r="AN8" s="90"/>
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A9" s="60"/>
+      <c r="A9" s="77"/>
       <c r="B9" s="23" t="s">
         <v>9</v>
       </c>
@@ -5778,7 +5754,7 @@
       <c r="T9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U9" s="60"/>
+      <c r="U9" s="77"/>
       <c r="V9" s="23" t="s">
         <v>9</v>
       </c>
@@ -5794,18 +5770,18 @@
       <c r="AE9" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF9" s="75"/>
-      <c r="AG9" s="76"/>
-      <c r="AH9" s="76"/>
-      <c r="AI9" s="76"/>
-      <c r="AJ9" s="76"/>
-      <c r="AK9" s="76"/>
-      <c r="AL9" s="76"/>
-      <c r="AM9" s="76"/>
-      <c r="AN9" s="77"/>
+      <c r="AF9" s="88"/>
+      <c r="AG9" s="89"/>
+      <c r="AH9" s="89"/>
+      <c r="AI9" s="89"/>
+      <c r="AJ9" s="89"/>
+      <c r="AK9" s="89"/>
+      <c r="AL9" s="89"/>
+      <c r="AM9" s="89"/>
+      <c r="AN9" s="90"/>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A10" s="60"/>
+      <c r="A10" s="77"/>
       <c r="B10" s="24" t="s">
         <v>32</v>
       </c>
@@ -5847,7 +5823,7 @@
       <c r="T10" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U10" s="60"/>
+      <c r="U10" s="77"/>
       <c r="V10" s="24" t="s">
         <v>32</v>
       </c>
@@ -5870,27 +5846,27 @@
       <c r="AE10" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="AF10" s="78"/>
-      <c r="AG10" s="79"/>
-      <c r="AH10" s="79"/>
-      <c r="AI10" s="79"/>
-      <c r="AJ10" s="79"/>
-      <c r="AK10" s="79"/>
-      <c r="AL10" s="79"/>
-      <c r="AM10" s="79"/>
-      <c r="AN10" s="80"/>
+      <c r="AF10" s="91"/>
+      <c r="AG10" s="92"/>
+      <c r="AH10" s="92"/>
+      <c r="AI10" s="92"/>
+      <c r="AJ10" s="92"/>
+      <c r="AK10" s="92"/>
+      <c r="AL10" s="92"/>
+      <c r="AM10" s="92"/>
+      <c r="AN10" s="93"/>
     </row>
     <row r="11" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="60" t="s">
+      <c r="A11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="B11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="62"/>
+      <c r="D11" s="76"/>
       <c r="E11" s="7" t="s">
         <v>45</v>
       </c>
@@ -5912,10 +5888,10 @@
       <c r="K11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L11" s="61" t="s">
+      <c r="L11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M11" s="62"/>
+      <c r="M11" s="76"/>
       <c r="N11" s="7" t="s">
         <v>45</v>
       </c>
@@ -5937,16 +5913,16 @@
       <c r="T11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U11" s="60" t="s">
+      <c r="U11" s="77" t="s">
         <v>53</v>
       </c>
       <c r="V11" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W11" s="61" t="s">
+      <c r="W11" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X11" s="62"/>
+      <c r="X11" s="76"/>
       <c r="Y11" s="7" t="s">
         <v>45</v>
       </c>
@@ -5968,90 +5944,90 @@
       <c r="AE11" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="AF11" s="72" t="s">
+      <c r="AF11" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="AG11" s="73"/>
-      <c r="AH11" s="73"/>
-      <c r="AI11" s="73"/>
-      <c r="AJ11" s="73"/>
-      <c r="AK11" s="73"/>
-      <c r="AL11" s="73"/>
-      <c r="AM11" s="73"/>
-      <c r="AN11" s="74"/>
+      <c r="AG11" s="86"/>
+      <c r="AH11" s="86"/>
+      <c r="AI11" s="86"/>
+      <c r="AJ11" s="86"/>
+      <c r="AK11" s="86"/>
+      <c r="AL11" s="86"/>
+      <c r="AM11" s="86"/>
+      <c r="AN11" s="87"/>
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A12" s="60"/>
+      <c r="A12" s="77"/>
       <c r="B12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="63">
-        <v>0</v>
-      </c>
-      <c r="D12" s="64"/>
+      <c r="C12" s="78">
+        <v>0</v>
+      </c>
+      <c r="D12" s="74"/>
       <c r="E12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F12" s="29"/>
-      <c r="G12" s="64">
-        <v>0</v>
-      </c>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64"/>
+      <c r="G12" s="74">
+        <v>0</v>
+      </c>
+      <c r="H12" s="74"/>
+      <c r="I12" s="74"/>
       <c r="J12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K12" s="30"/>
-      <c r="L12" s="63">
-        <v>0</v>
-      </c>
-      <c r="M12" s="64"/>
+      <c r="L12" s="78">
+        <v>0</v>
+      </c>
+      <c r="M12" s="74"/>
       <c r="N12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O12" s="29"/>
-      <c r="P12" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="64"/>
-      <c r="R12" s="64"/>
+      <c r="P12" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="74"/>
+      <c r="R12" s="74"/>
       <c r="S12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T12" s="30"/>
-      <c r="U12" s="60"/>
+      <c r="U12" s="77"/>
       <c r="V12" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W12" s="63">
-        <v>0</v>
-      </c>
-      <c r="X12" s="64"/>
+      <c r="W12" s="78">
+        <v>0</v>
+      </c>
+      <c r="X12" s="74"/>
       <c r="Y12" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z12" s="29"/>
-      <c r="AA12" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB12" s="64"/>
-      <c r="AC12" s="64"/>
+      <c r="AA12" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="74"/>
+      <c r="AC12" s="74"/>
       <c r="AD12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE12" s="30"/>
-      <c r="AF12" s="75"/>
-      <c r="AG12" s="76"/>
-      <c r="AH12" s="76"/>
-      <c r="AI12" s="76"/>
-      <c r="AJ12" s="76"/>
-      <c r="AK12" s="76"/>
-      <c r="AL12" s="76"/>
-      <c r="AM12" s="76"/>
-      <c r="AN12" s="77"/>
+      <c r="AF12" s="88"/>
+      <c r="AG12" s="89"/>
+      <c r="AH12" s="89"/>
+      <c r="AI12" s="89"/>
+      <c r="AJ12" s="89"/>
+      <c r="AK12" s="89"/>
+      <c r="AL12" s="89"/>
+      <c r="AM12" s="89"/>
+      <c r="AN12" s="90"/>
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A13" s="60"/>
+      <c r="A13" s="77"/>
       <c r="B13" s="23" t="s">
         <v>10</v>
       </c>
@@ -6106,7 +6082,7 @@
       <c r="T13" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U13" s="60"/>
+      <c r="U13" s="77"/>
       <c r="V13" s="23" t="s">
         <v>10</v>
       </c>
@@ -6134,18 +6110,18 @@
       <c r="AE13" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF13" s="75"/>
-      <c r="AG13" s="76"/>
-      <c r="AH13" s="76"/>
-      <c r="AI13" s="76"/>
-      <c r="AJ13" s="76"/>
-      <c r="AK13" s="76"/>
-      <c r="AL13" s="76"/>
-      <c r="AM13" s="76"/>
-      <c r="AN13" s="77"/>
+      <c r="AF13" s="88"/>
+      <c r="AG13" s="89"/>
+      <c r="AH13" s="89"/>
+      <c r="AI13" s="89"/>
+      <c r="AJ13" s="89"/>
+      <c r="AK13" s="89"/>
+      <c r="AL13" s="89"/>
+      <c r="AM13" s="89"/>
+      <c r="AN13" s="90"/>
     </row>
     <row r="14" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A14" s="60"/>
+      <c r="A14" s="77"/>
       <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
@@ -6176,7 +6152,7 @@
       <c r="T14" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U14" s="60"/>
+      <c r="U14" s="77"/>
       <c r="V14" s="23" t="s">
         <v>8</v>
       </c>
@@ -6192,18 +6168,18 @@
       <c r="AE14" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF14" s="75"/>
-      <c r="AG14" s="76"/>
-      <c r="AH14" s="76"/>
-      <c r="AI14" s="76"/>
-      <c r="AJ14" s="76"/>
-      <c r="AK14" s="76"/>
-      <c r="AL14" s="76"/>
-      <c r="AM14" s="76"/>
-      <c r="AN14" s="77"/>
+      <c r="AF14" s="88"/>
+      <c r="AG14" s="89"/>
+      <c r="AH14" s="89"/>
+      <c r="AI14" s="89"/>
+      <c r="AJ14" s="89"/>
+      <c r="AK14" s="89"/>
+      <c r="AL14" s="89"/>
+      <c r="AM14" s="89"/>
+      <c r="AN14" s="90"/>
     </row>
     <row r="15" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A15" s="60"/>
+      <c r="A15" s="77"/>
       <c r="B15" s="23" t="s">
         <v>37</v>
       </c>
@@ -6252,7 +6228,7 @@
       <c r="T15" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U15" s="60"/>
+      <c r="U15" s="77"/>
       <c r="V15" s="23" t="s">
         <v>37</v>
       </c>
@@ -6277,18 +6253,18 @@
       <c r="AE15" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF15" s="75"/>
-      <c r="AG15" s="76"/>
-      <c r="AH15" s="76"/>
-      <c r="AI15" s="76"/>
-      <c r="AJ15" s="76"/>
-      <c r="AK15" s="76"/>
-      <c r="AL15" s="76"/>
-      <c r="AM15" s="76"/>
-      <c r="AN15" s="77"/>
+      <c r="AF15" s="88"/>
+      <c r="AG15" s="89"/>
+      <c r="AH15" s="89"/>
+      <c r="AI15" s="89"/>
+      <c r="AJ15" s="89"/>
+      <c r="AK15" s="89"/>
+      <c r="AL15" s="89"/>
+      <c r="AM15" s="89"/>
+      <c r="AN15" s="90"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A16" s="60"/>
+      <c r="A16" s="77"/>
       <c r="B16" s="23" t="s">
         <v>9</v>
       </c>
@@ -6313,7 +6289,7 @@
       <c r="T16" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U16" s="60"/>
+      <c r="U16" s="77"/>
       <c r="V16" s="23" t="s">
         <v>9</v>
       </c>
@@ -6326,18 +6302,18 @@
       <c r="AE16" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF16" s="75"/>
-      <c r="AG16" s="76"/>
-      <c r="AH16" s="76"/>
-      <c r="AI16" s="76"/>
-      <c r="AJ16" s="76"/>
-      <c r="AK16" s="76"/>
-      <c r="AL16" s="76"/>
-      <c r="AM16" s="76"/>
-      <c r="AN16" s="77"/>
+      <c r="AF16" s="88"/>
+      <c r="AG16" s="89"/>
+      <c r="AH16" s="89"/>
+      <c r="AI16" s="89"/>
+      <c r="AJ16" s="89"/>
+      <c r="AK16" s="89"/>
+      <c r="AL16" s="89"/>
+      <c r="AM16" s="89"/>
+      <c r="AN16" s="90"/>
     </row>
     <row r="17" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A17" s="60"/>
+      <c r="A17" s="77"/>
       <c r="B17" s="24" t="s">
         <v>32</v>
       </c>
@@ -6377,7 +6353,7 @@
       <c r="T17" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U17" s="60"/>
+      <c r="U17" s="77"/>
       <c r="V17" s="24" t="s">
         <v>32</v>
       </c>
@@ -6398,27 +6374,27 @@
       <c r="AE17" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="AF17" s="78"/>
-      <c r="AG17" s="79"/>
-      <c r="AH17" s="79"/>
-      <c r="AI17" s="79"/>
-      <c r="AJ17" s="79"/>
-      <c r="AK17" s="79"/>
-      <c r="AL17" s="79"/>
-      <c r="AM17" s="79"/>
-      <c r="AN17" s="80"/>
+      <c r="AF17" s="91"/>
+      <c r="AG17" s="92"/>
+      <c r="AH17" s="92"/>
+      <c r="AI17" s="92"/>
+      <c r="AJ17" s="92"/>
+      <c r="AK17" s="92"/>
+      <c r="AL17" s="92"/>
+      <c r="AM17" s="92"/>
+      <c r="AN17" s="93"/>
     </row>
     <row r="18" spans="1:40" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="60" t="s">
+      <c r="A18" s="77" t="s">
         <v>72</v>
       </c>
       <c r="B18" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="62"/>
+      <c r="D18" s="76"/>
       <c r="E18" s="7" t="s">
         <v>45</v>
       </c>
@@ -6440,10 +6416,10 @@
       <c r="K18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="61" t="s">
+      <c r="L18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M18" s="62"/>
+      <c r="M18" s="76"/>
       <c r="N18" s="7" t="s">
         <v>45</v>
       </c>
@@ -6465,16 +6441,16 @@
       <c r="T18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U18" s="60" t="s">
+      <c r="U18" s="77" t="s">
         <v>72</v>
       </c>
       <c r="V18" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W18" s="61" t="s">
+      <c r="W18" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X18" s="62"/>
+      <c r="X18" s="76"/>
       <c r="Y18" s="7" t="s">
         <v>45</v>
       </c>
@@ -6496,90 +6472,90 @@
       <c r="AE18" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="AF18" s="72" t="s">
+      <c r="AF18" s="85" t="s">
         <v>47</v>
       </c>
-      <c r="AG18" s="73"/>
-      <c r="AH18" s="73"/>
-      <c r="AI18" s="73"/>
-      <c r="AJ18" s="73"/>
-      <c r="AK18" s="73"/>
-      <c r="AL18" s="73"/>
-      <c r="AM18" s="73"/>
-      <c r="AN18" s="74"/>
+      <c r="AG18" s="86"/>
+      <c r="AH18" s="86"/>
+      <c r="AI18" s="86"/>
+      <c r="AJ18" s="86"/>
+      <c r="AK18" s="86"/>
+      <c r="AL18" s="86"/>
+      <c r="AM18" s="86"/>
+      <c r="AN18" s="87"/>
     </row>
     <row r="19" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A19" s="60"/>
+      <c r="A19" s="77"/>
       <c r="B19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="63">
-        <v>0</v>
-      </c>
-      <c r="D19" s="64"/>
+      <c r="C19" s="78">
+        <v>0</v>
+      </c>
+      <c r="D19" s="74"/>
       <c r="E19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F19" s="29"/>
-      <c r="G19" s="64">
-        <v>0</v>
-      </c>
-      <c r="H19" s="64"/>
-      <c r="I19" s="64"/>
+      <c r="G19" s="74">
+        <v>0</v>
+      </c>
+      <c r="H19" s="74"/>
+      <c r="I19" s="74"/>
       <c r="J19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K19" s="30"/>
-      <c r="L19" s="63">
-        <v>0</v>
-      </c>
-      <c r="M19" s="64"/>
+      <c r="L19" s="78">
+        <v>0</v>
+      </c>
+      <c r="M19" s="74"/>
       <c r="N19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O19" s="29"/>
-      <c r="P19" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="64"/>
-      <c r="R19" s="64"/>
+      <c r="P19" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="74"/>
+      <c r="R19" s="74"/>
       <c r="S19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T19" s="30"/>
-      <c r="U19" s="60"/>
+      <c r="U19" s="77"/>
       <c r="V19" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W19" s="63">
-        <v>0</v>
-      </c>
-      <c r="X19" s="64"/>
+      <c r="W19" s="78">
+        <v>0</v>
+      </c>
+      <c r="X19" s="74"/>
       <c r="Y19" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z19" s="29"/>
-      <c r="AA19" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB19" s="64"/>
-      <c r="AC19" s="64"/>
+      <c r="AA19" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="74"/>
+      <c r="AC19" s="74"/>
       <c r="AD19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE19" s="30"/>
-      <c r="AF19" s="75"/>
-      <c r="AG19" s="76"/>
-      <c r="AH19" s="76"/>
-      <c r="AI19" s="76"/>
-      <c r="AJ19" s="76"/>
-      <c r="AK19" s="76"/>
-      <c r="AL19" s="76"/>
-      <c r="AM19" s="76"/>
-      <c r="AN19" s="77"/>
+      <c r="AF19" s="88"/>
+      <c r="AG19" s="89"/>
+      <c r="AH19" s="89"/>
+      <c r="AI19" s="89"/>
+      <c r="AJ19" s="89"/>
+      <c r="AK19" s="89"/>
+      <c r="AL19" s="89"/>
+      <c r="AM19" s="89"/>
+      <c r="AN19" s="90"/>
     </row>
     <row r="20" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A20" s="60"/>
+      <c r="A20" s="77"/>
       <c r="B20" s="23" t="s">
         <v>10</v>
       </c>
@@ -6637,7 +6613,7 @@
       <c r="T20" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U20" s="60"/>
+      <c r="U20" s="77"/>
       <c r="V20" s="23" t="s">
         <v>10</v>
       </c>
@@ -6668,18 +6644,18 @@
       <c r="AE20" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF20" s="75"/>
-      <c r="AG20" s="76"/>
-      <c r="AH20" s="76"/>
-      <c r="AI20" s="76"/>
-      <c r="AJ20" s="76"/>
-      <c r="AK20" s="76"/>
-      <c r="AL20" s="76"/>
-      <c r="AM20" s="76"/>
-      <c r="AN20" s="77"/>
+      <c r="AF20" s="88"/>
+      <c r="AG20" s="89"/>
+      <c r="AH20" s="89"/>
+      <c r="AI20" s="89"/>
+      <c r="AJ20" s="89"/>
+      <c r="AK20" s="89"/>
+      <c r="AL20" s="89"/>
+      <c r="AM20" s="89"/>
+      <c r="AN20" s="90"/>
     </row>
     <row r="21" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A21" s="60"/>
+      <c r="A21" s="77"/>
       <c r="B21" s="23" t="s">
         <v>8</v>
       </c>
@@ -6713,7 +6689,7 @@
       <c r="T21" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U21" s="60"/>
+      <c r="U21" s="77"/>
       <c r="V21" s="23" t="s">
         <v>8</v>
       </c>
@@ -6732,18 +6708,18 @@
       <c r="AE21" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF21" s="75"/>
-      <c r="AG21" s="76"/>
-      <c r="AH21" s="76"/>
-      <c r="AI21" s="76"/>
-      <c r="AJ21" s="76"/>
-      <c r="AK21" s="76"/>
-      <c r="AL21" s="76"/>
-      <c r="AM21" s="76"/>
-      <c r="AN21" s="77"/>
+      <c r="AF21" s="88"/>
+      <c r="AG21" s="89"/>
+      <c r="AH21" s="89"/>
+      <c r="AI21" s="89"/>
+      <c r="AJ21" s="89"/>
+      <c r="AK21" s="89"/>
+      <c r="AL21" s="89"/>
+      <c r="AM21" s="89"/>
+      <c r="AN21" s="90"/>
     </row>
     <row r="22" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A22" s="60"/>
+      <c r="A22" s="77"/>
       <c r="B22" s="23" t="s">
         <v>37</v>
       </c>
@@ -6795,7 +6771,7 @@
       <c r="T22" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U22" s="60"/>
+      <c r="U22" s="77"/>
       <c r="V22" s="23" t="s">
         <v>37</v>
       </c>
@@ -6823,18 +6799,18 @@
       <c r="AE22" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF22" s="75"/>
-      <c r="AG22" s="76"/>
-      <c r="AH22" s="76"/>
-      <c r="AI22" s="76"/>
-      <c r="AJ22" s="76"/>
-      <c r="AK22" s="76"/>
-      <c r="AL22" s="76"/>
-      <c r="AM22" s="76"/>
-      <c r="AN22" s="77"/>
+      <c r="AF22" s="88"/>
+      <c r="AG22" s="89"/>
+      <c r="AH22" s="89"/>
+      <c r="AI22" s="89"/>
+      <c r="AJ22" s="89"/>
+      <c r="AK22" s="89"/>
+      <c r="AL22" s="89"/>
+      <c r="AM22" s="89"/>
+      <c r="AN22" s="90"/>
     </row>
     <row r="23" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A23" s="60"/>
+      <c r="A23" s="77"/>
       <c r="B23" s="23" t="s">
         <v>9</v>
       </c>
@@ -6862,7 +6838,7 @@
       <c r="T23" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U23" s="60"/>
+      <c r="U23" s="77"/>
       <c r="V23" s="23" t="s">
         <v>9</v>
       </c>
@@ -6878,18 +6854,18 @@
       <c r="AE23" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="AF23" s="75"/>
-      <c r="AG23" s="76"/>
-      <c r="AH23" s="76"/>
-      <c r="AI23" s="76"/>
-      <c r="AJ23" s="76"/>
-      <c r="AK23" s="76"/>
-      <c r="AL23" s="76"/>
-      <c r="AM23" s="76"/>
-      <c r="AN23" s="77"/>
+      <c r="AF23" s="88"/>
+      <c r="AG23" s="89"/>
+      <c r="AH23" s="89"/>
+      <c r="AI23" s="89"/>
+      <c r="AJ23" s="89"/>
+      <c r="AK23" s="89"/>
+      <c r="AL23" s="89"/>
+      <c r="AM23" s="89"/>
+      <c r="AN23" s="90"/>
     </row>
     <row r="24" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A24" s="60"/>
+      <c r="A24" s="77"/>
       <c r="B24" s="24" t="s">
         <v>32</v>
       </c>
@@ -6931,7 +6907,7 @@
       <c r="T24" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U24" s="60"/>
+      <c r="U24" s="77"/>
       <c r="V24" s="24" t="s">
         <v>32</v>
       </c>
@@ -6954,27 +6930,27 @@
       <c r="AE24" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="AF24" s="78"/>
-      <c r="AG24" s="79"/>
-      <c r="AH24" s="79"/>
-      <c r="AI24" s="79"/>
-      <c r="AJ24" s="79"/>
-      <c r="AK24" s="79"/>
-      <c r="AL24" s="79"/>
-      <c r="AM24" s="79"/>
-      <c r="AN24" s="80"/>
+      <c r="AF24" s="91"/>
+      <c r="AG24" s="92"/>
+      <c r="AH24" s="92"/>
+      <c r="AI24" s="92"/>
+      <c r="AJ24" s="92"/>
+      <c r="AK24" s="92"/>
+      <c r="AL24" s="92"/>
+      <c r="AM24" s="92"/>
+      <c r="AN24" s="93"/>
     </row>
     <row r="25" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="77" t="s">
         <v>86</v>
       </c>
       <c r="B25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="D25" s="62"/>
+      <c r="D25" s="76"/>
       <c r="E25" s="7" t="s">
         <v>45</v>
       </c>
@@ -6996,10 +6972,10 @@
       <c r="K25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="L25" s="61" t="s">
+      <c r="L25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="M25" s="62"/>
+      <c r="M25" s="76"/>
       <c r="N25" s="7" t="s">
         <v>45</v>
       </c>
@@ -7021,16 +6997,16 @@
       <c r="T25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="U25" s="60" t="s">
+      <c r="U25" s="77" t="s">
         <v>86</v>
       </c>
       <c r="V25" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W25" s="61" t="s">
+      <c r="W25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="X25" s="62"/>
+      <c r="X25" s="76"/>
       <c r="Y25" s="7" t="s">
         <v>45</v>
       </c>
@@ -7052,10 +7028,10 @@
       <c r="AE25" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="AF25" s="61" t="s">
+      <c r="AF25" s="75" t="s">
         <v>48</v>
       </c>
-      <c r="AG25" s="62"/>
+      <c r="AG25" s="76"/>
       <c r="AH25" s="7" t="s">
         <v>45</v>
       </c>
@@ -7079,85 +7055,85 @@
       </c>
     </row>
     <row r="26" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A26" s="60"/>
+      <c r="A26" s="77"/>
       <c r="B26" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="63">
-        <v>0</v>
-      </c>
-      <c r="D26" s="64"/>
+      <c r="C26" s="78">
+        <v>0</v>
+      </c>
+      <c r="D26" s="74"/>
       <c r="E26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="F26" s="29"/>
-      <c r="G26" s="64">
-        <v>0</v>
-      </c>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
+      <c r="G26" s="74">
+        <v>0</v>
+      </c>
+      <c r="H26" s="74"/>
+      <c r="I26" s="74"/>
       <c r="J26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="K26" s="30"/>
-      <c r="L26" s="63">
-        <v>0</v>
-      </c>
-      <c r="M26" s="64"/>
+      <c r="L26" s="78">
+        <v>0</v>
+      </c>
+      <c r="M26" s="74"/>
       <c r="N26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="O26" s="29"/>
-      <c r="P26" s="64">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="64"/>
-      <c r="R26" s="64"/>
+      <c r="P26" s="74">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="74"/>
+      <c r="R26" s="74"/>
       <c r="S26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="T26" s="30"/>
-      <c r="U26" s="60"/>
+      <c r="U26" s="77"/>
       <c r="V26" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="W26" s="63">
-        <v>0</v>
-      </c>
-      <c r="X26" s="64"/>
+      <c r="W26" s="78">
+        <v>0</v>
+      </c>
+      <c r="X26" s="74"/>
       <c r="Y26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="Z26" s="29"/>
-      <c r="AA26" s="64">
-        <v>0</v>
-      </c>
-      <c r="AB26" s="64"/>
-      <c r="AC26" s="64"/>
+      <c r="AA26" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="74"/>
+      <c r="AC26" s="74"/>
       <c r="AD26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AE26" s="30"/>
-      <c r="AF26" s="63">
-        <v>0</v>
-      </c>
-      <c r="AG26" s="64"/>
+      <c r="AF26" s="78">
+        <v>0</v>
+      </c>
+      <c r="AG26" s="74"/>
       <c r="AH26" s="40" t="s">
         <v>52</v>
       </c>
       <c r="AI26" s="29"/>
-      <c r="AJ26" s="64">
-        <v>0</v>
-      </c>
-      <c r="AK26" s="64"/>
-      <c r="AL26" s="64"/>
+      <c r="AJ26" s="74">
+        <v>0</v>
+      </c>
+      <c r="AK26" s="74"/>
+      <c r="AL26" s="74"/>
       <c r="AM26" s="5" t="s">
         <v>46</v>
       </c>
       <c r="AN26" s="30"/>
     </row>
     <row r="27" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A27" s="60"/>
+      <c r="A27" s="77"/>
       <c r="B27" s="23" t="s">
         <v>10</v>
       </c>
@@ -7215,11 +7191,11 @@
       <c r="T27" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U27" s="60"/>
+      <c r="U27" s="77"/>
       <c r="V27" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="W27" s="56" t="s">
+      <c r="W27" s="48" t="s">
         <v>88</v>
       </c>
       <c r="X27" s="2" t="s">
@@ -7275,7 +7251,7 @@
       </c>
     </row>
     <row r="28" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A28" s="60"/>
+      <c r="A28" s="77"/>
       <c r="B28" s="23" t="s">
         <v>8</v>
       </c>
@@ -7309,7 +7285,7 @@
       <c r="T28" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U28" s="60"/>
+      <c r="U28" s="77"/>
       <c r="V28" s="23" t="s">
         <v>8</v>
       </c>
@@ -7345,7 +7321,7 @@
       </c>
     </row>
     <row r="29" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A29" s="60"/>
+      <c r="A29" s="77"/>
       <c r="B29" s="23" t="s">
         <v>37</v>
       </c>
@@ -7397,7 +7373,7 @@
       <c r="T29" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U29" s="60"/>
+      <c r="U29" s="77"/>
       <c r="V29" s="23" t="s">
         <v>37</v>
       </c>
@@ -7451,7 +7427,7 @@
       </c>
     </row>
     <row r="30" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A30" s="60"/>
+      <c r="A30" s="77"/>
       <c r="B30" s="23" t="s">
         <v>9</v>
       </c>
@@ -7479,7 +7455,7 @@
       <c r="T30" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="U30" s="60"/>
+      <c r="U30" s="77"/>
       <c r="V30" s="23" t="s">
         <v>9</v>
       </c>
@@ -7509,7 +7485,7 @@
       </c>
     </row>
     <row r="31" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A31" s="60"/>
+      <c r="A31" s="77"/>
       <c r="B31" s="24" t="s">
         <v>32</v>
       </c>
@@ -7551,7 +7527,7 @@
       <c r="T31" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="U31" s="60"/>
+      <c r="U31" s="77"/>
       <c r="V31" s="24" t="s">
         <v>32</v>
       </c>
@@ -7612,44 +7588,6 @@
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="AJ26:AL26"/>
-    <mergeCell ref="W19:X19"/>
-    <mergeCell ref="AA19:AC19"/>
-    <mergeCell ref="W18:X18"/>
-    <mergeCell ref="W25:X25"/>
-    <mergeCell ref="W26:X26"/>
-    <mergeCell ref="AA26:AC26"/>
-    <mergeCell ref="AF25:AG25"/>
-    <mergeCell ref="AF26:AG26"/>
-    <mergeCell ref="AF18:AN24"/>
-    <mergeCell ref="AF4:AN10"/>
-    <mergeCell ref="W12:X12"/>
-    <mergeCell ref="AA12:AC12"/>
-    <mergeCell ref="AF11:AN17"/>
-    <mergeCell ref="L18:M18"/>
-    <mergeCell ref="L11:M11"/>
-    <mergeCell ref="AA5:AC5"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="P19:R19"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="L12:M12"/>
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="L25:M25"/>
-    <mergeCell ref="L26:M26"/>
-    <mergeCell ref="P26:R26"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="P5:R5"/>
-    <mergeCell ref="W5:X5"/>
     <mergeCell ref="A18:A24"/>
     <mergeCell ref="U18:U24"/>
     <mergeCell ref="A25:A31"/>
@@ -7666,6 +7604,44 @@
     <mergeCell ref="A11:A17"/>
     <mergeCell ref="U11:U17"/>
     <mergeCell ref="L5:M5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="W5:X5"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L26:M26"/>
+    <mergeCell ref="P26:R26"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="P19:R19"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="AF4:AN10"/>
+    <mergeCell ref="W12:X12"/>
+    <mergeCell ref="AA12:AC12"/>
+    <mergeCell ref="AF11:AN17"/>
+    <mergeCell ref="L18:M18"/>
+    <mergeCell ref="L11:M11"/>
+    <mergeCell ref="AA5:AC5"/>
+    <mergeCell ref="AJ26:AL26"/>
+    <mergeCell ref="W19:X19"/>
+    <mergeCell ref="AA19:AC19"/>
+    <mergeCell ref="W18:X18"/>
+    <mergeCell ref="W25:X25"/>
+    <mergeCell ref="W26:X26"/>
+    <mergeCell ref="AA26:AC26"/>
+    <mergeCell ref="AF25:AG25"/>
+    <mergeCell ref="AF26:AG26"/>
+    <mergeCell ref="AF18:AN24"/>
   </mergeCells>
   <pageMargins left="0.19685039370078741" right="0.11811023622047245" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -7690,27 +7666,27 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="95" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="98" t="s">
+      <c r="A3" s="61" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="99"/>
-      <c r="D3" s="97" t="s">
+      <c r="C3" s="65"/>
+      <c r="D3" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="97"/>
-      <c r="F3" s="97"/>
-      <c r="G3" s="92" t="s">
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="93"/>
-      <c r="I3" s="93"/>
-      <c r="J3" s="94"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="60"/>
     </row>
     <row r="4" spans="1:10" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="96"/>
+      <c r="A4" s="62"/>
       <c r="B4" s="10" t="s">
         <v>15</v>
       </c>
@@ -7740,7 +7716,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="100" t="s">
+      <c r="A5" s="66" t="s">
         <v>51</v>
       </c>
       <c r="B5" s="16" t="s">
@@ -7772,43 +7748,43 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="101"/>
-      <c r="B6" s="103" t="s">
+      <c r="A6" s="67"/>
+      <c r="B6" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="C6" s="104"/>
-      <c r="D6" s="103" t="s">
+      <c r="C6" s="70"/>
+      <c r="D6" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="E6" s="104"/>
-      <c r="F6" s="105"/>
-      <c r="G6" s="103" t="s">
+      <c r="E6" s="70"/>
+      <c r="F6" s="71"/>
+      <c r="G6" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="H6" s="104"/>
-      <c r="I6" s="104"/>
-      <c r="J6" s="105"/>
+      <c r="H6" s="70"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="71"/>
     </row>
     <row r="7" spans="1:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="102"/>
-      <c r="B7" s="89" t="s">
+      <c r="A7" s="68"/>
+      <c r="B7" s="55" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="91"/>
-      <c r="D7" s="89" t="s">
+      <c r="C7" s="56"/>
+      <c r="D7" s="55" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="90"/>
-      <c r="F7" s="91"/>
-      <c r="G7" s="89" t="s">
+      <c r="E7" s="57"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="H7" s="90"/>
-      <c r="I7" s="90"/>
-      <c r="J7" s="91"/>
+      <c r="H7" s="57"/>
+      <c r="I7" s="57"/>
+      <c r="J7" s="56"/>
     </row>
     <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="81" t="s">
+      <c r="A8" s="49" t="s">
         <v>55</v>
       </c>
       <c r="B8" s="43" t="s">
@@ -7840,43 +7816,43 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="82"/>
-      <c r="B9" s="84" t="s">
+      <c r="A9" s="50"/>
+      <c r="B9" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="85"/>
-      <c r="D9" s="84" t="s">
+      <c r="C9" s="53"/>
+      <c r="D9" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="86"/>
-      <c r="F9" s="85"/>
-      <c r="G9" s="84" t="s">
+      <c r="E9" s="54"/>
+      <c r="F9" s="53"/>
+      <c r="G9" s="52" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="86"/>
-      <c r="I9" s="86"/>
-      <c r="J9" s="85"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="53"/>
     </row>
     <row r="10" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="83"/>
-      <c r="B10" s="89" t="s">
+      <c r="A10" s="51"/>
+      <c r="B10" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="91"/>
-      <c r="D10" s="89" t="s">
+      <c r="C10" s="56"/>
+      <c r="D10" s="55" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="90"/>
-      <c r="F10" s="91"/>
-      <c r="G10" s="89" t="s">
+      <c r="E10" s="57"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="55" t="s">
         <v>70</v>
       </c>
-      <c r="H10" s="90"/>
-      <c r="I10" s="90"/>
-      <c r="J10" s="91"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="57"/>
+      <c r="J10" s="56"/>
     </row>
     <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="81" t="s">
+      <c r="A11" s="49" t="s">
         <v>73</v>
       </c>
       <c r="B11" s="43" t="s">
@@ -7908,43 +7884,43 @@
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="82"/>
-      <c r="B12" s="84" t="s">
+      <c r="A12" s="50"/>
+      <c r="B12" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="C12" s="85"/>
-      <c r="D12" s="84" t="s">
+      <c r="C12" s="53"/>
+      <c r="D12" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="86"/>
-      <c r="F12" s="85"/>
-      <c r="G12" s="84" t="s">
+      <c r="E12" s="54"/>
+      <c r="F12" s="53"/>
+      <c r="G12" s="52" t="s">
         <v>85</v>
       </c>
-      <c r="H12" s="86"/>
-      <c r="I12" s="86"/>
-      <c r="J12" s="85"/>
+      <c r="H12" s="54"/>
+      <c r="I12" s="54"/>
+      <c r="J12" s="53"/>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="83"/>
-      <c r="B13" s="89" t="s">
+      <c r="A13" s="51"/>
+      <c r="B13" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="C13" s="91"/>
-      <c r="D13" s="89" t="s">
+      <c r="C13" s="56"/>
+      <c r="D13" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="E13" s="90"/>
-      <c r="F13" s="91"/>
-      <c r="G13" s="89" t="s">
+      <c r="E13" s="57"/>
+      <c r="F13" s="56"/>
+      <c r="G13" s="55" t="s">
         <v>84</v>
       </c>
-      <c r="H13" s="90"/>
-      <c r="I13" s="90"/>
-      <c r="J13" s="91"/>
+      <c r="H13" s="57"/>
+      <c r="I13" s="57"/>
+      <c r="J13" s="56"/>
     </row>
     <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="81" t="s">
+      <c r="A14" s="49" t="s">
         <v>73</v>
       </c>
       <c r="B14" s="43" t="s">
@@ -7976,57 +7952,50 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="82"/>
-      <c r="B15" s="84" t="s">
+      <c r="A15" s="50"/>
+      <c r="B15" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="85"/>
-      <c r="D15" s="84" t="s">
+      <c r="C15" s="53"/>
+      <c r="D15" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="E15" s="86"/>
-      <c r="F15" s="85"/>
-      <c r="G15" s="84" t="s">
+      <c r="E15" s="54"/>
+      <c r="F15" s="53"/>
+      <c r="G15" s="52" t="s">
         <v>102</v>
       </c>
-      <c r="H15" s="86"/>
-      <c r="I15" s="86"/>
-      <c r="J15" s="85"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="53"/>
     </row>
     <row r="16" spans="1:10" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="83"/>
-      <c r="B16" s="87" t="s">
+      <c r="A16" s="51"/>
+      <c r="B16" s="72" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="88"/>
-      <c r="D16" s="89" t="s">
+      <c r="C16" s="73"/>
+      <c r="D16" s="55" t="s">
         <v>91</v>
       </c>
-      <c r="E16" s="90"/>
-      <c r="F16" s="91"/>
-      <c r="G16" s="89" t="s">
+      <c r="E16" s="57"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="55" t="s">
         <v>92</v>
       </c>
-      <c r="H16" s="90"/>
-      <c r="I16" s="90"/>
-      <c r="J16" s="91"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="G13:J13"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="A14:A16"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G15:J15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="G16:J16"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="D3:F3"/>
@@ -8038,13 +8007,20 @@
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="G6:J6"/>
     <mergeCell ref="G7:J7"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:J15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:J16"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="G12:J12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="G13:J13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>

</xml_diff>